<commit_message>
refit sim to final N20/3216 skeleton + lock exact drivetrain spec in BOM
config+xml: 60mm wheels (r=0.03), 0.11 track, MAX_WHEEL_RAD_S 25.05, round chassis, actuator force = real 100:1 N20 stall torque, low wheel damping so torque (not drag) caps speed. Verified: 0.59 m/s fwd, 6.0 rad/s yaw, 49 tests pass. BOM: Pololu HPCB 6V 100:1 extended-shaft + encoder, 60mm wheel, 2S V_batt-comp wiring.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/phase2/roybot-BOM.xlsx
+++ b/docs/phase2/roybot-BOM.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Tools" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BOM'!$A$8:$I$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BOM'!$A$8:$I$46</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="H4" s="4">
-        <f>SUMIF(A9:A45,"Purchased",H9:H45)</f>
+        <f>SUMIF(A9:A46,"Purchased",H9:H46)</f>
         <v/>
       </c>
     </row>
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="H5" s="5">
-        <f>SUMIF(A9:A45,"To buy",H9:H45)</f>
+        <f>SUMIF(A9:A46,"To buy",H9:H46)</f>
         <v/>
       </c>
     </row>
@@ -564,7 +564,7 @@
         </is>
       </c>
       <c r="H6" s="6">
-        <f>SUM(H9:H45)</f>
+        <f>SUM(H9:H46)</f>
         <v/>
       </c>
     </row>
@@ -818,7 +818,7 @@
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>N20 gearmotor w/ magnetic encoder, 6 V</t>
+          <t>Pololu HPCB 6V 100:1 micro metal gearmotor, EXTENDED back-shaft</t>
         </is>
       </c>
       <c r="D14" s="8" t="n">
@@ -826,7 +826,7 @@
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>Final drivetrain: closed-loop speed + odometry (needed for docking). Pick gear ratio for speed/torque</t>
+          <t>Verified pick: ~239 rpm loaded -&gt; 0.75 m/s top @60mm wheel, 1.6 kg-cm stall. EXTENDED shaft is REQUIRED so the encoder mounts on the rear</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="G14" s="10" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="H14" s="10">
         <f>D14*G14</f>
@@ -856,24 +856,24 @@
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>N20 motor bracket / mount</t>
+          <t>Pololu magnetic quadrature encoder pair (micro metal gearmotor)</t>
         </is>
       </c>
       <c r="D15" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>Mount N20s to the 3216 frame - likely needs a small printed adapter to fit the frame's hole pattern</t>
+          <t>Hall A/B, 12 CPR/motor-rev -&gt; 1200 CPR/wheel-rev at 100:1 (already x4-decoded; do NOT x4 again). VCC = 3.3V</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>Pololu / Amazon</t>
+          <t>Pololu</t>
         </is>
       </c>
       <c r="G15" s="10" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H15" s="10">
         <f>D15*G15</f>
@@ -894,7 +894,7 @@
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>Wheel for N20 (3 mm D-shaft), ~60 mm</t>
+          <t>N20 motor bracket / mount</t>
         </is>
       </c>
       <c r="D16" s="8" t="n">
@@ -902,7 +902,7 @@
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>The 3216 wheels don't fit the N20 shaft</t>
+          <t>Mount N20s to the 3216 frame - likely needs a small printed adapter to fit the frame's hole pattern</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="G16" s="10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H16" s="10">
         <f>D16*G16</f>
@@ -932,24 +932,24 @@
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>TB6612FNG dual H-bridge breakout</t>
+          <t>Wheel for N20 (3 mm D-shaft), 60 mm OD</t>
         </is>
       </c>
       <c r="D17" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>Motor driver (efficient; chosen over DRV8833/L298N)</t>
+          <t>60mm chosen so loaded top speed lands at 0.75 m/s (65mm overshoots). 3216 wheels don't fit the N20 shaft</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>Adafruit / Pololu</t>
+          <t>Pololu / Amazon</t>
         </is>
       </c>
       <c r="G17" s="10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H17" s="10">
         <f>D17*G17</f>
@@ -965,12 +965,12 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Sensors</t>
+          <t>Drivetrain</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>MPU-6050 IMU</t>
+          <t>TB6612FNG dual H-bridge breakout</t>
         </is>
       </c>
       <c r="D18" s="8" t="n">
@@ -978,16 +978,16 @@
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>Roll/pitch + tip/stall reflexes; proprioception for the policy</t>
+          <t>Motor driver. Run 2S via firmware V_batt duty comp (~6V avg), PWM &gt;=20kHz, encoder-static stall cutoff</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Adafruit / Pololu</t>
         </is>
       </c>
       <c r="G18" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H18" s="10">
         <f>D18*G18</f>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>OV5647 camera (Pi-compatible)</t>
+          <t>MPU-6050 IMU</t>
         </is>
       </c>
       <c r="D19" s="8" t="n">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>Cat tracking (perception, #2)</t>
+          <t>Roll/pitch + tip/stall reflexes; proprioception for the policy</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -1025,7 +1025,7 @@
         </is>
       </c>
       <c r="G19" s="10" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H19" s="10">
         <f>D19*G19</f>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>Pi Zero CSI ribbon (mini -&gt; standard)</t>
+          <t>OV5647 camera (Pi-compatible)</t>
         </is>
       </c>
       <c r="D20" s="8" t="n">
@@ -1054,16 +1054,16 @@
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>Pi Zero needs the narrow CSI cable</t>
+          <t>Cat tracking (perception, #2)</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>Adafruit</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G20" s="10" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="H20" s="10">
         <f>D20*G20</f>
@@ -1084,24 +1084,24 @@
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>IR reflectance cliff/edge sensor</t>
+          <t>Pi Zero CSI ribbon (mini -&gt; standard)</t>
         </is>
       </c>
       <c r="D21" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>Edge detect -&gt; back off (safety floor). Stops falls off tables/stairs</t>
+          <t>Pi Zero needs the narrow CSI cable</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Adafruit</t>
         </is>
       </c>
       <c r="G21" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H21" s="10">
         <f>D21*G21</f>
@@ -1122,7 +1122,7 @@
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Bump microswitch (lever)</t>
+          <t>IR reflectance cliff/edge sensor</t>
         </is>
       </c>
       <c r="D22" s="8" t="n">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>Front bump detect -&gt; back off</t>
+          <t>Edge detect -&gt; back off (safety floor). Stops falls off tables/stairs</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -1139,7 +1139,7 @@
         </is>
       </c>
       <c r="G22" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H22" s="10">
         <f>D22*G22</f>
@@ -1155,20 +1155,20 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Audio</t>
+          <t>Sensors</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>INMP441 I2S microphone</t>
+          <t>Bump microswitch (lever)</t>
         </is>
       </c>
       <c r="D23" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>Wake-word / voice in (#5)</t>
+          <t>Front bump detect -&gt; back off</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -1177,7 +1177,7 @@
         </is>
       </c>
       <c r="G23" s="10" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H23" s="10">
         <f>D23*G23</f>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>MAX98357A I2S amplifier</t>
+          <t>INMP441 I2S microphone</t>
         </is>
       </c>
       <c r="D24" s="8" t="n">
@@ -1206,16 +1206,16 @@
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>Speaker driver (voice reports #5)</t>
+          <t>Wake-word / voice in (#5)</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
-          <t>Adafruit</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G24" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H24" s="10">
         <f>D24*G24</f>
@@ -1236,7 +1236,7 @@
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>Speaker 4-8 ohm (small)</t>
+          <t>MAX98357A I2S amplifier</t>
         </is>
       </c>
       <c r="D25" s="8" t="n">
@@ -1244,16 +1244,16 @@
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>Audio out</t>
+          <t>Speaker driver (voice reports #5)</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Adafruit</t>
         </is>
       </c>
       <c r="G25" s="10" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H25" s="10">
         <f>D25*G25</f>
@@ -1269,12 +1269,12 @@
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>Expression</t>
+          <t>Audio</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>WS2812 RGB LED ring</t>
+          <t>Speaker 4-8 ohm (small)</t>
         </is>
       </c>
       <c r="D26" s="8" t="n">
@@ -1282,7 +1282,7 @@
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>Expressive 'personality' output</t>
+          <t>Audio out</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
@@ -1291,7 +1291,7 @@
         </is>
       </c>
       <c r="G26" s="10" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H26" s="10">
         <f>D26*G26</f>
@@ -1307,12 +1307,12 @@
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>Expression</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>LiPo battery 2S 7.4 V (small)</t>
+          <t>WS2812 RGB LED ring</t>
         </is>
       </c>
       <c r="D27" s="8" t="n">
@@ -1320,16 +1320,16 @@
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>Main power for the 6 V N20s (PWM-limited). Couples to the charger/BMS choice</t>
+          <t>Expressive 'personality' output</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
-          <t>HobbyKing / Amazon</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G27" s="10" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H27" s="10">
         <f>D27*G27</f>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>5 V buck regulator (3 A)</t>
+          <t>LiPo battery 2S 7.4 V (small)</t>
         </is>
       </c>
       <c r="D28" s="8" t="n">
@@ -1358,16 +1358,16 @@
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>Dedicated Pi rail; isolates Pi from motor surges</t>
+          <t>Main power for the 6 V N20s (PWM-limited). Couples to the charger/BMS choice</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
-          <t>Pololu / Amazon</t>
+          <t>HobbyKing / Amazon</t>
         </is>
       </c>
       <c r="G28" s="10" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="H28" s="10">
         <f>D28*G28</f>
@@ -1388,24 +1388,24 @@
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>Bulk capacitor 470-1000 uF</t>
+          <t>5 V buck regulator (3 A)</t>
         </is>
       </c>
       <c r="D29" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>Brownout protection (Pi + motor rails)</t>
+          <t>Dedicated Pi rail; isolates Pi from motor surges</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Pololu / Amazon</t>
         </is>
       </c>
       <c r="G29" s="10" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H29" s="10">
         <f>D29*G29</f>
@@ -1426,15 +1426,15 @@
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>2S LiPo BMS / protection + charge board</t>
+          <t>Bulk capacitor 470-1000 uF</t>
         </is>
       </c>
       <c r="D30" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>Safe charge/discharge; this is the on-bot side of docking</t>
+          <t>Brownout protection (Pi + motor rails)</t>
         </is>
       </c>
       <c r="F30" s="8" t="inlineStr">
@@ -1443,7 +1443,7 @@
         </is>
       </c>
       <c r="G30" s="10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H30" s="10">
         <f>D30*G30</f>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>XT30 / JST battery connector set</t>
+          <t>2S LiPo BMS / protection + charge board</t>
         </is>
       </c>
       <c r="D31" s="8" t="n">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>Battery + charge connectors</t>
+          <t>Safe charge/discharge; this is the on-bot side of docking</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
@@ -1481,7 +1481,7 @@
         </is>
       </c>
       <c r="G31" s="10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H31" s="10">
         <f>D31*G31</f>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>Inline fuse + holder</t>
+          <t>XT30 / JST battery connector set</t>
         </is>
       </c>
       <c r="D32" s="8" t="n">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>Battery short protection</t>
+          <t>Battery + charge connectors</t>
         </is>
       </c>
       <c r="F32" s="8" t="inlineStr">
@@ -1519,7 +1519,7 @@
         </is>
       </c>
       <c r="G32" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H32" s="10">
         <f>D32*G32</f>
@@ -1540,7 +1540,7 @@
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>Power switch (SPST)</t>
+          <t>Inline fuse + holder</t>
         </is>
       </c>
       <c r="D33" s="8" t="n">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>Main cutoff</t>
+          <t>Battery short protection</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
@@ -1573,12 +1573,12 @@
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>Dock</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>Pogo-pin charging contacts (bot + dock pair)</t>
+          <t>Power switch (SPST)</t>
         </is>
       </c>
       <c r="D34" s="8" t="n">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>Spring-pin charge contacts for self-docking</t>
+          <t>Main cutoff</t>
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="G34" s="10" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H34" s="10">
         <f>D34*G34</f>
@@ -1616,7 +1616,7 @@
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>TSOP38238 IR receiver</t>
+          <t>Pogo-pin charging contacts (bot + dock pair)</t>
         </is>
       </c>
       <c r="D35" s="8" t="n">
@@ -1624,7 +1624,7 @@
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>On the bot: IR homing to the dock</t>
+          <t>Spring-pin charge contacts for self-docking</t>
         </is>
       </c>
       <c r="F35" s="8" t="inlineStr">
@@ -1633,7 +1633,7 @@
         </is>
       </c>
       <c r="G35" s="10" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H35" s="10">
         <f>D35*G35</f>
@@ -1654,7 +1654,7 @@
       </c>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>IR LED beacon + driver</t>
+          <t>TSOP38238 IR receiver</t>
         </is>
       </c>
       <c r="D36" s="8" t="n">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>On the dock: homing beacon</t>
+          <t>On the bot: IR homing to the dock</t>
         </is>
       </c>
       <c r="F36" s="8" t="inlineStr">
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="G36" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H36" s="10">
         <f>D36*G36</f>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>Dock PSU (5 V / 2 A) + barrel jack</t>
+          <t>IR LED beacon + driver</t>
         </is>
       </c>
       <c r="D37" s="8" t="n">
@@ -1700,7 +1700,7 @@
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>Powers the charging dock</t>
+          <t>On the dock: homing beacon</t>
         </is>
       </c>
       <c r="F37" s="8" t="inlineStr">
@@ -1709,7 +1709,7 @@
         </is>
       </c>
       <c r="G37" s="10" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H37" s="10">
         <f>D37*G37</f>
@@ -1730,7 +1730,7 @@
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>Dock base + alignment funnel (PETG print)</t>
+          <t>Dock PSU (5 V / 2 A) + barrel jack</t>
         </is>
       </c>
       <c r="D38" s="8" t="n">
@@ -1738,16 +1738,16 @@
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>Passive funnel; printed</t>
+          <t>Powers the charging dock</t>
         </is>
       </c>
       <c r="F38" s="8" t="inlineStr">
         <is>
-          <t>(PETG)</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G38" s="10" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H38" s="10">
         <f>D38*G38</f>
@@ -1763,12 +1763,12 @@
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>Cat-safety</t>
+          <t>Dock</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>Captive lure (feather/pom on short rigid/braided arm)</t>
+          <t>Dock base + alignment funnel (PETG print)</t>
         </is>
       </c>
       <c r="D39" s="8" t="n">
@@ -1776,16 +1776,16 @@
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>#1 hazard control: NO free end, over-molded. No loose string ever</t>
+          <t>Passive funnel; printed</t>
         </is>
       </c>
       <c r="F39" s="8" t="inlineStr">
         <is>
-          <t>craft + over-mold</t>
+          <t>(PETG)</t>
         </is>
       </c>
       <c r="G39" s="10" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H39" s="10">
         <f>D39*G39</f>
@@ -1801,12 +1801,12 @@
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>Structure</t>
+          <t>Cat-safety</t>
         </is>
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>PETG filament (known-safe) spool</t>
+          <t>Captive lure (feather/pom on short rigid/braided arm)</t>
         </is>
       </c>
       <c r="D40" s="8" t="n">
@@ -1814,16 +1814,16 @@
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>Cover / wheel shroud / lure boom / dock funnel / N20 adapter prints</t>
+          <t>#1 hazard control: NO free end, over-molded. No loose string ever</t>
         </is>
       </c>
       <c r="F40" s="8" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>craft + over-mold</t>
         </is>
       </c>
       <c r="G40" s="10" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="H40" s="10">
         <f>D40*G40</f>
@@ -1844,7 +1844,7 @@
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>Heat-set inserts + screws</t>
+          <t>PETG filament (known-safe) spool</t>
         </is>
       </c>
       <c r="D41" s="8" t="n">
@@ -1852,7 +1852,7 @@
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>Tool-locked battery hatch; captive fasteners</t>
+          <t>Cover / wheel shroud / lure boom / dock funnel / N20 adapter prints</t>
         </is>
       </c>
       <c r="F41" s="8" t="inlineStr">
@@ -1861,7 +1861,7 @@
         </is>
       </c>
       <c r="G41" s="10" t="n">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="H41" s="10">
         <f>D41*G41</f>
@@ -1877,12 +1877,12 @@
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>Wiring</t>
+          <t>Structure</t>
         </is>
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>Silicone hookup wire (assorted AWG)</t>
+          <t>Heat-set inserts + screws</t>
         </is>
       </c>
       <c r="D42" s="8" t="n">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>Motor + logic wiring</t>
+          <t>Tool-locked battery hatch; captive fasteners</t>
         </is>
       </c>
       <c r="F42" s="8" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>JST / Dupont connector kit</t>
+          <t>Silicone hookup wire (assorted AWG)</t>
         </is>
       </c>
       <c r="D43" s="8" t="n">
@@ -1928,7 +1928,7 @@
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>Removable connections</t>
+          <t>Motor + logic wiring</t>
         </is>
       </c>
       <c r="F43" s="8" t="inlineStr">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="G43" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H43" s="10">
         <f>D43*G43</f>
@@ -1958,7 +1958,7 @@
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>Standoffs / M2.5 hardware kit</t>
+          <t>JST / Dupont connector kit</t>
         </is>
       </c>
       <c r="D44" s="8" t="n">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>Mount Pi + boards to the chassis</t>
+          <t>Removable connections</t>
         </is>
       </c>
       <c r="F44" s="8" t="inlineStr">
@@ -1996,7 +1996,7 @@
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>Heat-shrink assortment</t>
+          <t>Standoffs / M2.5 hardware kit</t>
         </is>
       </c>
       <c r="D45" s="8" t="n">
@@ -2004,7 +2004,7 @@
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>Insulation</t>
+          <t>Mount Pi + boards to the chassis</t>
         </is>
       </c>
       <c r="F45" s="8" t="inlineStr">
@@ -2013,7 +2013,7 @@
         </is>
       </c>
       <c r="G45" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H45" s="10">
         <f>D45*G45</f>
@@ -2021,13 +2021,51 @@
       </c>
       <c r="I45" s="8" t="inlineStr"/>
     </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>To buy</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>Heat-shrink assortment</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" s="9" t="inlineStr">
+        <is>
+          <t>Insulation</t>
+        </is>
+      </c>
+      <c r="F46" s="8" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G46" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="H46" s="10">
+        <f>D46*G46</f>
+        <v/>
+      </c>
+      <c r="I46" s="8" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A8:I45"/>
+  <autoFilter ref="A8:I46"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A9:A45">
+  <conditionalFormatting sqref="A9:A46">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Purchased"</formula>
     </cfRule>
@@ -2036,7 +2074,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="A9:A45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A9:A46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Purchased,To buy"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>